<commit_message>
Update Customer Intelligence dashboard
</commit_message>
<xml_diff>
--- a/MOCK DATA.xlsx
+++ b/MOCK DATA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranthihoanganh/Downloads/Customer Intelligence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FD7589-2FCF-CA46-B973-D5A22C42CE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE6AC40-2E0F-0845-8F64-BEB6AEE36838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="47">
   <si>
     <t>MCOK</t>
   </si>
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -257,12 +257,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -272,6 +266,13 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -527,18 +528,18 @@
       <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="7">
-        <v>32000</v>
-      </c>
-      <c r="E2" s="8">
-        <v>0</v>
-      </c>
-      <c r="F2" s="8">
-        <v>1</v>
-      </c>
-      <c r="G2" s="9">
+      <c r="D2" s="5">
+        <v>7500</v>
+      </c>
+      <c r="E2" s="6">
+        <v>0</v>
+      </c>
+      <c r="F2" s="6">
+        <v>1</v>
+      </c>
+      <c r="G2" s="7">
         <f xml:space="preserve"> D2/SUM(D2,D5,D8,D11,D14)</f>
-        <v>0.29090909090909089</v>
+        <v>0.23809523809523808</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="26.75" customHeight="1">
@@ -549,16 +550,16 @@
       <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="7">
-        <v>0</v>
-      </c>
-      <c r="E3" s="8">
-        <v>0</v>
-      </c>
-      <c r="F3" s="8">
-        <v>1</v>
-      </c>
-      <c r="G3" s="9">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0</v>
+      </c>
+      <c r="F3" s="6">
+        <v>1</v>
+      </c>
+      <c r="G3" s="7">
         <f>D3/SUM(D3,D6,D9,D12,D15)</f>
         <v>0</v>
       </c>
@@ -571,18 +572,18 @@
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="7">
-        <v>8000</v>
-      </c>
-      <c r="E4" s="8">
-        <v>0</v>
-      </c>
-      <c r="F4" s="8">
-        <v>1</v>
-      </c>
-      <c r="G4" s="9">
+      <c r="D4" s="5">
+        <v>3000</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7">
         <f>D4/SUM(D4,D7,D10,D13,D16)</f>
-        <v>0.13333333333333333</v>
+        <v>0.13043478260869565</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="26.75" customHeight="1">
@@ -593,18 +594,18 @@
       <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="7">
-        <v>24000</v>
-      </c>
-      <c r="E5" s="8">
-        <v>0</v>
-      </c>
-      <c r="F5" s="8">
-        <v>1</v>
-      </c>
-      <c r="G5" s="9">
+      <c r="D5" s="5">
+        <v>8000</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7">
         <f>D5/SUM(D2,D5,D8,D11,D14)</f>
-        <v>0.21818181818181817</v>
+        <v>0.25396825396825395</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="26.75" customHeight="1">
@@ -615,18 +616,18 @@
       <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="7">
-        <v>4000</v>
-      </c>
-      <c r="E6" s="8">
-        <v>0</v>
-      </c>
-      <c r="F6" s="8">
-        <v>1</v>
-      </c>
-      <c r="G6" s="9">
+      <c r="D6" s="5">
+        <v>3000</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7">
         <f>D6/SUM(D3,D6,D9,D12,D15)</f>
-        <v>0.27586206896551724</v>
+        <v>0.35294117647058826</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="26.75" customHeight="1">
@@ -637,18 +638,18 @@
       <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="7">
-        <v>18000</v>
-      </c>
-      <c r="E7" s="8">
-        <v>0</v>
-      </c>
-      <c r="F7" s="8">
-        <v>1</v>
-      </c>
-      <c r="G7" s="9">
+      <c r="D7" s="5">
+        <v>7000</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6">
+        <v>1</v>
+      </c>
+      <c r="G7" s="7">
         <f>D7/SUM(D4,D7,D10,D13,D16)</f>
-        <v>0.3</v>
+        <v>0.30434782608695654</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="26.75" customHeight="1">
@@ -659,18 +660,18 @@
       <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="7">
-        <v>28000</v>
-      </c>
-      <c r="E8" s="8">
-        <v>0</v>
-      </c>
-      <c r="F8" s="8">
-        <v>1</v>
-      </c>
-      <c r="G8" s="9">
+      <c r="D8" s="5">
+        <v>10000</v>
+      </c>
+      <c r="E8" s="6">
+        <v>0</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7">
         <f>D8/SUM(D2,D5,D8,D11,D14)</f>
-        <v>0.25454545454545452</v>
+        <v>0.31746031746031744</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="26.75" customHeight="1">
@@ -681,18 +682,18 @@
       <c r="C9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="7">
-        <v>5500</v>
-      </c>
-      <c r="E9" s="8">
-        <v>0</v>
-      </c>
-      <c r="F9" s="8">
-        <v>1</v>
-      </c>
-      <c r="G9" s="9">
+      <c r="D9" s="5">
+        <v>2000</v>
+      </c>
+      <c r="E9" s="6">
+        <v>0</v>
+      </c>
+      <c r="F9" s="6">
+        <v>1</v>
+      </c>
+      <c r="G9" s="7">
         <f xml:space="preserve"> D9/SUM(D3,D6,D9,D12,D15)</f>
-        <v>0.37931034482758619</v>
+        <v>0.23529411764705882</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="26.75" customHeight="1">
@@ -703,18 +704,18 @@
       <c r="C10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="7">
-        <v>12000</v>
-      </c>
-      <c r="E10" s="8">
-        <v>0</v>
-      </c>
-      <c r="F10" s="8">
-        <v>1</v>
-      </c>
-      <c r="G10" s="9">
+      <c r="D10" s="5">
+        <v>3000</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6">
+        <v>1</v>
+      </c>
+      <c r="G10" s="7">
         <f>D10/SUM(D4,D7,D10,D13,D16)</f>
-        <v>0.2</v>
+        <v>0.13043478260869565</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="26.75" customHeight="1">
@@ -725,18 +726,18 @@
       <c r="C11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="7">
-        <v>18000</v>
-      </c>
-      <c r="E11" s="8">
-        <v>0</v>
-      </c>
-      <c r="F11" s="8">
-        <v>1</v>
-      </c>
-      <c r="G11" s="9">
+      <c r="D11" s="5">
+        <v>3000</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7">
         <f>D11/SUM(D2,D5,D8,D11,D14)</f>
-        <v>0.16363636363636364</v>
+        <v>9.5238095238095233E-2</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="26.75" customHeight="1">
@@ -747,18 +748,18 @@
       <c r="C12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="7">
-        <v>3500</v>
-      </c>
-      <c r="E12" s="8">
-        <v>0</v>
-      </c>
-      <c r="F12" s="8">
-        <v>1</v>
-      </c>
-      <c r="G12" s="9">
+      <c r="D12" s="5">
+        <v>2000</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6">
+        <v>1</v>
+      </c>
+      <c r="G12" s="7">
         <f xml:space="preserve"> D12 / SUM(D3,D6,D9,D12,D15)</f>
-        <v>0.2413793103448276</v>
+        <v>0.23529411764705882</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="26.75" customHeight="1">
@@ -769,18 +770,18 @@
       <c r="C13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="7">
-        <v>16000</v>
-      </c>
-      <c r="E13" s="8">
-        <v>0</v>
-      </c>
-      <c r="F13" s="8">
-        <v>1</v>
-      </c>
-      <c r="G13" s="9">
+      <c r="D13" s="5">
+        <v>4000</v>
+      </c>
+      <c r="E13" s="6">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6">
+        <v>1</v>
+      </c>
+      <c r="G13" s="7">
         <f xml:space="preserve"> D13 / SUM(D4,D7,D10,D13,D16)</f>
-        <v>0.26666666666666666</v>
+        <v>0.17391304347826086</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="26.75" customHeight="1">
@@ -791,18 +792,18 @@
       <c r="C14" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="7">
-        <v>8000</v>
-      </c>
-      <c r="E14" s="8">
-        <v>0</v>
-      </c>
-      <c r="F14" s="8">
-        <v>1</v>
-      </c>
-      <c r="G14" s="9">
+      <c r="D14" s="5">
+        <v>3000</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7">
         <f>D14/SUM(D2,D5,D8,D11,D14)</f>
-        <v>7.2727272727272724E-2</v>
+        <v>9.5238095238095233E-2</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="26.75" customHeight="1">
@@ -813,18 +814,18 @@
       <c r="C15" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="5">
         <v>1500</v>
       </c>
-      <c r="E15" s="8">
-        <v>0</v>
-      </c>
-      <c r="F15" s="8">
-        <v>1</v>
-      </c>
-      <c r="G15" s="9">
+      <c r="E15" s="6">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7">
         <f xml:space="preserve"> D15/ SUM(D3,D6,D9,D12,D15)</f>
-        <v>0.10344827586206896</v>
+        <v>0.17647058823529413</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="26.75" customHeight="1">
@@ -835,195 +836,189 @@
       <c r="C16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="5">
         <v>6000</v>
       </c>
-      <c r="E16" s="8">
-        <v>0</v>
-      </c>
-      <c r="F16" s="8">
-        <v>1</v>
-      </c>
-      <c r="G16" s="9">
+      <c r="E16" s="6">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7">
         <f>D16/SUM(D4,D7,D10,D13,D16)</f>
-        <v>0.1</v>
+        <v>0.2608695652173913</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="A17" s="3"/>
       <c r="B17" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="7">
-        <v>70000</v>
-      </c>
-      <c r="E17" s="8">
-        <v>1</v>
-      </c>
-      <c r="F17" s="8">
-        <v>2</v>
-      </c>
-      <c r="G17" s="9">
-        <f xml:space="preserve"> D17 /SUM(D17,D21)</f>
-        <v>0.88607594936708856</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="D17" s="5">
+        <v>25000</v>
+      </c>
+      <c r="E17" s="6">
+        <v>1</v>
+      </c>
+      <c r="F17" s="6">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7"/>
     </row>
     <row r="18" spans="1:7" ht="26.75" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="7">
-        <v>18000</v>
-      </c>
-      <c r="E18" s="8">
-        <v>1</v>
-      </c>
-      <c r="F18" s="8">
-        <v>2</v>
-      </c>
-      <c r="G18" s="9">
-        <f xml:space="preserve"> D18/SUM(D18,D22)</f>
-        <v>0.78260869565217395</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D18" s="5">
+        <v>20000</v>
+      </c>
+      <c r="E18" s="6">
+        <v>1</v>
+      </c>
+      <c r="F18" s="6">
+        <v>1</v>
+      </c>
+      <c r="G18" s="7"/>
     </row>
     <row r="19" spans="1:7" ht="26.75" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="7">
-        <v>12000</v>
-      </c>
-      <c r="E19" s="8">
-        <v>1</v>
-      </c>
-      <c r="F19" s="8">
-        <v>2</v>
-      </c>
-      <c r="G19" s="9">
-        <f xml:space="preserve"> D19/SUM(D19,D23)</f>
-        <v>0.8</v>
+        <v>10</v>
+      </c>
+      <c r="D19" s="5">
+        <v>10000</v>
+      </c>
+      <c r="E19" s="6">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6">
+        <v>1</v>
+      </c>
+      <c r="G19" s="10">
+        <v>0.26</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A20" s="3"/>
+      <c r="A20" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="B20" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" s="7">
-        <v>10000</v>
-      </c>
-      <c r="E20" s="8">
-        <v>1</v>
-      </c>
-      <c r="F20" s="8">
-        <v>2</v>
-      </c>
-      <c r="G20" s="9">
-        <f>D20/SUM(D20,D26)</f>
-        <v>0.45454545454545453</v>
+        <v>17</v>
+      </c>
+      <c r="D20" s="5">
+        <v>25000</v>
+      </c>
+      <c r="E20" s="6">
+        <v>1</v>
+      </c>
+      <c r="F20" s="6">
+        <v>2</v>
+      </c>
+      <c r="G20" s="7">
+        <f xml:space="preserve"> D20 /SUM(D20,D24)</f>
+        <v>0.78125</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="26.75" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" s="7">
-        <v>9000</v>
-      </c>
-      <c r="E21" s="8">
-        <v>1</v>
-      </c>
-      <c r="F21" s="8">
-        <v>2</v>
-      </c>
-      <c r="G21" s="9">
-        <f xml:space="preserve"> D21/SUM(D17,D21)</f>
-        <v>0.11392405063291139</v>
+        <v>18</v>
+      </c>
+      <c r="D21" s="5">
+        <v>15000</v>
+      </c>
+      <c r="E21" s="6">
+        <v>1</v>
+      </c>
+      <c r="F21" s="6">
+        <v>2</v>
+      </c>
+      <c r="G21" s="7">
+        <f xml:space="preserve"> D21/SUM(D21,D25)</f>
+        <v>0.78947368421052633</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="26.75" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="7">
-        <v>5000</v>
-      </c>
-      <c r="E22" s="8">
-        <v>1</v>
-      </c>
-      <c r="F22" s="8">
-        <v>2</v>
-      </c>
-      <c r="G22" s="9">
-        <f xml:space="preserve"> D22/SUM(D22,D18)</f>
-        <v>0.21739130434782608</v>
+        <v>19</v>
+      </c>
+      <c r="D22" s="5">
+        <v>10000</v>
+      </c>
+      <c r="E22" s="6">
+        <v>1</v>
+      </c>
+      <c r="F22" s="6">
+        <v>2</v>
+      </c>
+      <c r="G22" s="7">
+        <f xml:space="preserve"> D22/SUM(D22,D26)</f>
+        <v>0.76923076923076927</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="26.75" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" s="7">
-        <v>3000</v>
-      </c>
-      <c r="E23" s="8">
-        <v>1</v>
-      </c>
-      <c r="F23" s="8">
-        <v>2</v>
-      </c>
-      <c r="G23" s="9">
-        <f xml:space="preserve"> D23/SUM(D23,D19)</f>
-        <v>0.2</v>
+        <v>20</v>
+      </c>
+      <c r="D23" s="5">
+        <v>2000</v>
+      </c>
+      <c r="E23" s="6">
+        <v>1</v>
+      </c>
+      <c r="F23" s="6">
+        <v>2</v>
+      </c>
+      <c r="G23" s="7">
+        <f>D23/SUM(D23,D29)</f>
+        <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="26.75" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="7">
-        <v>4000</v>
-      </c>
-      <c r="E24" s="8">
-        <v>1</v>
-      </c>
-      <c r="F24" s="8">
-        <v>2</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>46</v>
+        <v>17</v>
+      </c>
+      <c r="D24" s="5">
+        <v>7000</v>
+      </c>
+      <c r="E24" s="6">
+        <v>1</v>
+      </c>
+      <c r="F24" s="6">
+        <v>2</v>
+      </c>
+      <c r="G24" s="7">
+        <f xml:space="preserve"> D24/SUM(D20,D24)</f>
+        <v>0.21875</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="26.75" customHeight="1">
@@ -1032,19 +1027,20 @@
         <v>11</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D25" s="7">
-        <v>15000</v>
-      </c>
-      <c r="E25" s="8">
-        <v>1</v>
-      </c>
-      <c r="F25" s="8">
-        <v>2</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>46</v>
+        <v>18</v>
+      </c>
+      <c r="D25" s="5">
+        <v>4000</v>
+      </c>
+      <c r="E25" s="6">
+        <v>1</v>
+      </c>
+      <c r="F25" s="6">
+        <v>2</v>
+      </c>
+      <c r="G25" s="7">
+        <f xml:space="preserve"> D25/SUM(D25,D21)</f>
+        <v>0.21052631578947367</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="26.75" customHeight="1">
@@ -1053,381 +1049,445 @@
         <v>11</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D26" s="7">
-        <v>12000</v>
-      </c>
-      <c r="E26" s="8">
-        <v>1</v>
-      </c>
-      <c r="F26" s="8">
-        <v>2</v>
-      </c>
-      <c r="G26" s="9">
-        <f xml:space="preserve"> D26/SUM(D20,D26)</f>
-        <v>0.54545454545454541</v>
+        <v>19</v>
+      </c>
+      <c r="D26" s="5">
+        <v>3000</v>
+      </c>
+      <c r="E26" s="6">
+        <v>1</v>
+      </c>
+      <c r="F26" s="6">
+        <v>2</v>
+      </c>
+      <c r="G26" s="7">
+        <f xml:space="preserve"> D26/SUM(D26,D22)</f>
+        <v>0.23076923076923078</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A27" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A27" s="3"/>
       <c r="B27" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D27" s="7">
-        <v>10000</v>
-      </c>
-      <c r="E27" s="8">
-        <v>2</v>
-      </c>
-      <c r="F27" s="8">
-        <v>3</v>
-      </c>
-      <c r="G27" s="9">
-        <f xml:space="preserve"> D27/SUM(D17,D21)</f>
-        <v>0.12658227848101267</v>
+        <v>21</v>
+      </c>
+      <c r="D27" s="5">
+        <v>4000</v>
+      </c>
+      <c r="E27" s="6">
+        <v>1</v>
+      </c>
+      <c r="F27" s="6">
+        <v>2</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="26.75" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="3" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D28" s="7">
-        <v>8000</v>
-      </c>
-      <c r="E28" s="8">
-        <v>2</v>
-      </c>
-      <c r="F28" s="8">
-        <v>3</v>
-      </c>
-      <c r="G28" s="9">
-        <f xml:space="preserve"> D28/SUM(D18,D22)</f>
-        <v>0.34782608695652173</v>
+        <v>22</v>
+      </c>
+      <c r="D28" s="5">
+        <v>7500</v>
+      </c>
+      <c r="E28" s="6">
+        <v>1</v>
+      </c>
+      <c r="F28" s="6">
+        <v>2</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="26.75" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="3" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D29" s="7">
-        <v>8000</v>
-      </c>
-      <c r="E29" s="8">
-        <v>2</v>
-      </c>
-      <c r="F29" s="8">
-        <v>3</v>
-      </c>
-      <c r="G29" s="9">
-        <f xml:space="preserve"> D29/SUM(D19,D23)</f>
-        <v>0.53333333333333333</v>
+        <v>20</v>
+      </c>
+      <c r="D29" s="5">
+        <v>12000</v>
+      </c>
+      <c r="E29" s="6">
+        <v>1</v>
+      </c>
+      <c r="F29" s="6">
+        <v>2</v>
+      </c>
+      <c r="G29" s="7">
+        <f xml:space="preserve"> D29/SUM(D23,D29)</f>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A30" s="3"/>
+      <c r="A30" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="B30" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D30" s="7">
-        <v>1900</v>
-      </c>
-      <c r="E30" s="8">
-        <v>2</v>
-      </c>
-      <c r="F30" s="8">
+      <c r="D30" s="5">
+        <v>8000</v>
+      </c>
+      <c r="E30" s="6">
+        <v>2</v>
+      </c>
+      <c r="F30" s="6">
         <v>3</v>
       </c>
-      <c r="G30" s="9">
-        <f xml:space="preserve"> D30/D24</f>
-        <v>0.47499999999999998</v>
+      <c r="G30" s="7">
+        <f xml:space="preserve"> D30/SUM(D20,D24)</f>
+        <v>0.25</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="26.75" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D31" s="7">
-        <v>2000</v>
-      </c>
-      <c r="E31" s="8">
-        <v>2</v>
-      </c>
-      <c r="F31" s="8">
+      <c r="D31" s="5">
+        <v>5000</v>
+      </c>
+      <c r="E31" s="6">
+        <v>2</v>
+      </c>
+      <c r="F31" s="6">
         <v>3</v>
       </c>
-      <c r="G31" s="9">
-        <f>D31/D25</f>
-        <v>0.13333333333333333</v>
+      <c r="G31" s="7">
+        <f xml:space="preserve"> D31/SUM(D21,D25)</f>
+        <v>0.26315789473684209</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="26.75" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D32" s="7">
-        <v>1800</v>
-      </c>
-      <c r="E32" s="8">
-        <v>2</v>
-      </c>
-      <c r="F32" s="8">
+      <c r="D32" s="5">
+        <v>5000</v>
+      </c>
+      <c r="E32" s="6">
+        <v>2</v>
+      </c>
+      <c r="F32" s="6">
         <v>3</v>
       </c>
-      <c r="G32" s="9">
-        <f>D32/SUM(D26,D20)</f>
-        <v>8.1818181818181818E-2</v>
+      <c r="G32" s="7">
+        <f xml:space="preserve"> D32/SUM(D22,D26)</f>
+        <v>0.38461538461538464</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A33" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D33" s="7">
-        <v>8350</v>
-      </c>
-      <c r="E33" s="8">
+      <c r="D33" s="5">
+        <v>1900</v>
+      </c>
+      <c r="E33" s="6">
+        <v>2</v>
+      </c>
+      <c r="F33" s="6">
         <v>3</v>
       </c>
-      <c r="F33" s="8">
-        <v>4</v>
-      </c>
-      <c r="G33" s="9">
-        <f>D33/SUM(D27:D32)</f>
-        <v>0.26340694006309151</v>
+      <c r="G33" s="7">
+        <f xml:space="preserve"> D33/D27</f>
+        <v>0.47499999999999998</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="26.75" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D34" s="7">
-        <v>4320</v>
-      </c>
-      <c r="E34" s="8">
-        <v>4</v>
-      </c>
-      <c r="F34" s="8">
-        <v>5</v>
-      </c>
-      <c r="G34" s="9">
-        <f>D34/D33</f>
-        <v>0.51736526946107786</v>
+        <v>24</v>
+      </c>
+      <c r="D34" s="5">
+        <v>2000</v>
+      </c>
+      <c r="E34" s="6">
+        <v>2</v>
+      </c>
+      <c r="F34" s="6">
+        <v>3</v>
+      </c>
+      <c r="G34" s="7">
+        <f>D34/D28</f>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A35" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="A35" s="3"/>
       <c r="B35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D35" s="7">
-        <v>7580</v>
-      </c>
-      <c r="E35" s="8">
+      <c r="D35" s="5">
+        <v>1800</v>
+      </c>
+      <c r="E35" s="6">
+        <v>2</v>
+      </c>
+      <c r="F35" s="6">
         <v>3</v>
       </c>
-      <c r="F35" s="8">
-        <v>5</v>
-      </c>
-      <c r="G35" s="9">
-        <f>D35/SUM(D27:D32)</f>
-        <v>0.2391167192429022</v>
+      <c r="G35" s="7">
+        <f>D35/SUM(D29,D23)</f>
+        <v>0.12857142857142856</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="26.75" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D36" s="7">
-        <v>9150</v>
-      </c>
-      <c r="E36" s="8">
-        <v>5</v>
-      </c>
-      <c r="F36" s="8">
-        <v>6</v>
-      </c>
-      <c r="G36" s="9">
-        <f>D36/SUM(D34:D35)</f>
-        <v>0.76890756302521013</v>
+        <v>26</v>
+      </c>
+      <c r="D36" s="5">
+        <v>8350</v>
+      </c>
+      <c r="E36" s="6">
+        <v>3</v>
+      </c>
+      <c r="F36" s="6">
+        <v>4</v>
+      </c>
+      <c r="G36" s="7">
+        <f>D36/SUM(D30:D35)</f>
+        <v>0.35232067510548526</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="26.75" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D37" s="7">
-        <v>2380</v>
-      </c>
-      <c r="E37" s="8">
+      <c r="D37" s="5">
+        <v>4320</v>
+      </c>
+      <c r="E37" s="6">
+        <v>4</v>
+      </c>
+      <c r="F37" s="6">
         <v>5</v>
       </c>
-      <c r="F37" s="8">
-        <v>6</v>
-      </c>
-      <c r="G37" s="9">
-        <f>D37/SUM(D34:D35)</f>
-        <v>0.2</v>
+      <c r="G37" s="7">
+        <f>D37/D36</f>
+        <v>0.51736526946107786</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A38" s="3"/>
+      <c r="A38" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="B38" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" s="7">
-        <v>360</v>
-      </c>
-      <c r="E38" s="8">
+      <c r="D38" s="5">
+        <v>7580</v>
+      </c>
+      <c r="E38" s="6">
+        <v>3</v>
+      </c>
+      <c r="F38" s="6">
         <v>5</v>
       </c>
-      <c r="F38" s="8">
-        <v>6</v>
-      </c>
-      <c r="G38" s="9">
-        <f xml:space="preserve"> D38/SUM(D34:D35)</f>
-        <v>3.0252100840336135E-2</v>
+      <c r="G38" s="7">
+        <f>D38/SUM(D30:D35)</f>
+        <v>0.31983122362869199</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="26.75" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D39" s="7">
-        <v>120</v>
-      </c>
-      <c r="E39" s="8">
+      <c r="D39" s="5">
+        <v>9150</v>
+      </c>
+      <c r="E39" s="6">
+        <v>5</v>
+      </c>
+      <c r="F39" s="6">
         <v>6</v>
       </c>
-      <c r="F39" s="8">
-        <v>7</v>
-      </c>
-      <c r="G39" s="9">
-        <f>D39/D36</f>
-        <v>1.3114754098360656E-2</v>
+      <c r="G39" s="7">
+        <f>D39/SUM(D37:D38)</f>
+        <v>0.76890756302521013</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="26.75" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D40" s="7">
-        <v>7450</v>
-      </c>
-      <c r="E40" s="8">
+        <v>32</v>
+      </c>
+      <c r="D40" s="5">
+        <v>2380</v>
+      </c>
+      <c r="E40" s="6">
+        <v>5</v>
+      </c>
+      <c r="F40" s="6">
         <v>6</v>
       </c>
-      <c r="F40" s="8">
-        <v>7</v>
-      </c>
-      <c r="G40" s="9">
-        <f>D40/D36</f>
-        <v>0.81420765027322406</v>
+      <c r="G40" s="7">
+        <f>D40/SUM(D37:D38)</f>
+        <v>0.2</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="26.75" customHeight="1">
       <c r="A41" s="3"/>
       <c r="B41" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D41" s="7">
-        <v>1560</v>
-      </c>
-      <c r="E41" s="8">
+        <v>33</v>
+      </c>
+      <c r="D41" s="5">
+        <v>360</v>
+      </c>
+      <c r="E41" s="6">
+        <v>5</v>
+      </c>
+      <c r="F41" s="6">
         <v>6</v>
       </c>
-      <c r="F41" s="8">
-        <v>7</v>
-      </c>
-      <c r="G41" s="9">
-        <f>D41/D36</f>
-        <v>0.17049180327868851</v>
+      <c r="G41" s="7">
+        <f xml:space="preserve"> D41/SUM(D37:D38)</f>
+        <v>3.0252100840336135E-2</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="26.75" customHeight="1">
-      <c r="A42" s="3"/>
+      <c r="A42" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="B42" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C42" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D42" s="5">
+        <v>120</v>
+      </c>
+      <c r="E42" s="6">
+        <v>6</v>
+      </c>
+      <c r="F42" s="6">
+        <v>7</v>
+      </c>
+      <c r="G42" s="7">
+        <f>D42/D39</f>
+        <v>1.3114754098360656E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="26.75" customHeight="1">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D43" s="5">
+        <v>7450</v>
+      </c>
+      <c r="E43" s="6">
+        <v>6</v>
+      </c>
+      <c r="F43" s="6">
+        <v>7</v>
+      </c>
+      <c r="G43" s="7">
+        <f>D43/D39</f>
+        <v>0.81420765027322406</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="26.75" customHeight="1">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D44" s="5">
+        <v>1560</v>
+      </c>
+      <c r="E44" s="6">
+        <v>6</v>
+      </c>
+      <c r="F44" s="6">
+        <v>7</v>
+      </c>
+      <c r="G44" s="7">
+        <f>D44/D39</f>
+        <v>0.17049180327868851</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="26.75" customHeight="1">
+      <c r="A45" s="3"/>
+      <c r="B45" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D42" s="7">
+      <c r="D45" s="5">
         <v>1250</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E45" s="6">
         <v>6</v>
       </c>
-      <c r="F42" s="8">
+      <c r="F45" s="6">
         <v>7</v>
       </c>
-      <c r="G42" s="9">
-        <f>D42/D36</f>
+      <c r="G45" s="7">
+        <f>D45/D39</f>
         <v>0.13661202185792351</v>
       </c>
     </row>
@@ -1449,10 +1509,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="6"/>
+      <c r="B1" s="9"/>
     </row>
     <row r="2" spans="1:2" ht="15">
       <c r="A2" s="4" t="s">

</xml_diff>